<commit_message>
New Prompt, New Evaluation Grid
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vincent Dusanek\Documents\GitHub\ai-rater-prompts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290F7149-D201-4670-8BEE-FF750DBEAE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E4283B-1466-4202-AD7D-9BF491A452CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4E8083B-D79D-4448-92F1-4C454AB4E1C3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <r>
       <rPr>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t>Textfeld</t>
+  </si>
+  <si>
+    <t>Id</t>
   </si>
 </sst>
 </file>
@@ -615,30 +618,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D6E467-3641-4C92-A3EE-80450D709D04}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="113.42578125" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="113.42578125" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:2" ht="371.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:3" ht="371.25" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:2" ht="303.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:3" ht="303.75" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>